<commit_message>
Update unit mismatches data files for transactions and materials
- Removed outdated entries from unit-mismatches.csv for transactions to enhance data accuracy.
- Updated binary content of unit-mismatches.xlsx files for both materials and transactions to reflect the latest changes.
</commit_message>
<xml_diff>
--- a/data/materials/_unit-mismatches/unit-mismatches.xlsx
+++ b/data/materials/_unit-mismatches/unit-mismatches.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>المصدر</t>
   </si>
@@ -27,27 +27,12 @@
   <si>
     <t>الوحدة في ملف الجرد</t>
   </si>
-  <si>
-    <t>مواد خام</t>
-  </si>
-  <si>
-    <t>11006002</t>
-  </si>
-  <si>
-    <t>عود بلاستيك تثبيت الجوان محلى</t>
-  </si>
-  <si>
-    <t>عدد</t>
-  </si>
-  <si>
-    <t>متر</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -59,10 +44,6 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -106,16 +87,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -459,7 +434,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -486,25 +461,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E2"/>
+  <autoFilter ref="A1:E1"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>